<commit_message>
Clean up unused imports in AppointmentController
Removed several unused import statements from AppointmentController.java to improve code readability and maintainability. No functional changes were made.
</commit_message>
<xml_diff>
--- a/Helper.xlsx
+++ b/Helper.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23025" windowHeight="9660"/>
+    <workbookView windowWidth="28800" windowHeight="12180" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="API's" sheetId="2" r:id="rId2"/>
+    <sheet name="API's Pending" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="177">
   <si>
     <t>Command to connect localhost to internet URL</t>
   </si>
@@ -53,6 +53,532 @@
   </si>
   <si>
     <t>MY_SECRET_KEY_123456</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>API Endpoint</t>
+  </si>
+  <si>
+    <t>HTTP Method</t>
+  </si>
+  <si>
+    <t>Parameters</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>/auth/doctor/register</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>Body: userName, userEmail, userPassword, role, firstName, lastName, licenseNumber, phone, specialization, qualifications, location, language, experience, availability, consultationFees, ratings, availabilityStarting, availabilityEnd</t>
+  </si>
+  <si>
+    <t>/auth/patient/register</t>
+  </si>
+  <si>
+    <t>Body: userName, userEmail, userPassword, role, firstName, lastName, dateOfBirth, gender, phoneNumber, address, emergencyPhoneNumber</t>
+  </si>
+  <si>
+    <t>/auth/admin/register</t>
+  </si>
+  <si>
+    <t>Body: userName, userEmail, userPassword, role, firstName, lastName, department, accessLevel</t>
+  </si>
+  <si>
+    <t>/auth/login</t>
+  </si>
+  <si>
+    <t>Body: userName, userPassword</t>
+  </si>
+  <si>
+    <t>/auth/logout</t>
+  </si>
+  <si>
+    <t>No parameters</t>
+  </si>
+  <si>
+    <t>Doctor</t>
+  </si>
+  <si>
+    <t>/doctor/all</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>/doctor/{id}</t>
+  </si>
+  <si>
+    <t>Path: id (Long)</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>/doctor/search</t>
+  </si>
+  <si>
+    <t>Body: specialization, location, language, minExperience, maxExperience</t>
+  </si>
+  <si>
+    <t>/doctor/filter</t>
+  </si>
+  <si>
+    <t>Body: availability, consultationFees, ratings</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}/schedule</t>
+  </si>
+  <si>
+    <t>Path: doctorId (Long), Query: weekStart (yyyy-MM-dd)</t>
+  </si>
+  <si>
+    <t>/doctor/availability</t>
+  </si>
+  <si>
+    <t>Body: doctor (object reference), availableDate, startTime, endTime, isBooked (optional)</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}/availability</t>
+  </si>
+  <si>
+    <t>Path: doctorId (Long)</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}/appointments</t>
+  </si>
+  <si>
+    <t>Appointments</t>
+  </si>
+  <si>
+    <t>/appointments/doctor</t>
+  </si>
+  <si>
+    <t>Body: doctorId, patientId, availabilityId, appointmentDate, startTime, endTime, appointmentType, status, paymentStatus, consultationFee, symptoms, notes</t>
+  </si>
+  <si>
+    <t>/appointments/patient</t>
+  </si>
+  <si>
+    <t>Body: doctorId, patientId, availabilityId, appointmentDate, startTime, endTime, appointmentType, symptoms</t>
+  </si>
+  <si>
+    <t>/appointments/cancel</t>
+  </si>
+  <si>
+    <t>Body: appointmentId, cancellationReason, cancelledBy, cancelledAt</t>
+  </si>
+  <si>
+    <t>Patient</t>
+  </si>
+  <si>
+    <t>/patient/all</t>
+  </si>
+  <si>
+    <t>/patient/{id}</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>/user/all</t>
+  </si>
+  <si>
+    <t>/user/{id}</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>/admin/all</t>
+  </si>
+  <si>
+    <t>/admin/{id}</t>
+  </si>
+  <si>
+    <t>Medical Records</t>
+  </si>
+  <si>
+    <t>/medical-records/upload/{patientId}</t>
+  </si>
+  <si>
+    <t>Path: patientId (Long), Form-data: file (MultipartFile), notes (String, optional)</t>
+  </si>
+  <si>
+    <t>/medical-records/patient/{patientId}</t>
+  </si>
+  <si>
+    <t>Path: patientId (Long)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14.05"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Summary Statistics</t>
+    </r>
+  </si>
+  <si>
+    <t>Total Endpoints</t>
+  </si>
+  <si>
+    <t>POST Requests</t>
+  </si>
+  <si>
+    <t>GET Requests</t>
+  </si>
+  <si>
+    <t>DELETE Requests</t>
+  </si>
+  <si>
+    <t>Endpoint</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>Due Date</t>
+  </si>
+  <si>
+    <t>Request Body / Parameters (Demo)</t>
+  </si>
+  <si>
+    <t>/auth/refresh-token</t>
+  </si>
+  <si>
+    <t>Generate new access token</t>
+  </si>
+  <si>
+    <t>PENDING</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>{"refreshToken":"xxxx"}</t>
+  </si>
+  <si>
+    <t>/auth/change-password</t>
+  </si>
+  <si>
+    <t>User changes password</t>
+  </si>
+  <si>
+    <t>{"oldPassword":"", "newPassword":""}</t>
+  </si>
+  <si>
+    <t>/auth/forgot-password</t>
+  </si>
+  <si>
+    <t>Send OTP/link</t>
+  </si>
+  <si>
+    <t>{"email":""}</t>
+  </si>
+  <si>
+    <t>/auth/reset-password</t>
+  </si>
+  <si>
+    <t>Reset password using OTP</t>
+  </si>
+  <si>
+    <t>{"otp":"", "newPassword":""}</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}</t>
+  </si>
+  <si>
+    <t>Update doctor profile</t>
+  </si>
+  <si>
+    <t>{"name":"", "specialization":"", "experience":""}</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}/schedule/{slotId}</t>
+  </si>
+  <si>
+    <t>Update schedule slot</t>
+  </si>
+  <si>
+    <t>{"startTime":"", "endTime":""}</t>
+  </si>
+  <si>
+    <t>Delete schedule slot</t>
+  </si>
+  <si>
+    <t>Path Variable: doctorId, slotId</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}/appointments/upcoming</t>
+  </si>
+  <si>
+    <t>Get upcoming appointments</t>
+  </si>
+  <si>
+    <t>Path Variable: doctorId</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}/appointments/past</t>
+  </si>
+  <si>
+    <t>Get past appointments</t>
+  </si>
+  <si>
+    <t>/doctor/{doctorId}/reviews</t>
+  </si>
+  <si>
+    <t>Add review</t>
+  </si>
+  <si>
+    <t>{"rating":5, "comment":""}</t>
+  </si>
+  <si>
+    <t>Get reviews</t>
+  </si>
+  <si>
+    <t>/patient/{patientId}</t>
+  </si>
+  <si>
+    <t>Update patient info</t>
+  </si>
+  <si>
+    <t>{"name":"", "age":""}</t>
+  </si>
+  <si>
+    <t>Delete patient</t>
+  </si>
+  <si>
+    <t>Path Variable: patientId</t>
+  </si>
+  <si>
+    <t>/patient/{patientId}/appointments</t>
+  </si>
+  <si>
+    <t>Get appointment history</t>
+  </si>
+  <si>
+    <t>/patient/{patientId}/doctors</t>
+  </si>
+  <si>
+    <t>Get consulted doctors list</t>
+  </si>
+  <si>
+    <t>/patient/{patientId}/medical-records</t>
+  </si>
+  <si>
+    <t>Get medical record summary</t>
+  </si>
+  <si>
+    <t>/appointments/book</t>
+  </si>
+  <si>
+    <t>Book appointment</t>
+  </si>
+  <si>
+    <t>{"doctorId":"", "patientId":"", "date":"", "time":""}</t>
+  </si>
+  <si>
+    <t>/appointments/{appointmentId}/reschedule</t>
+  </si>
+  <si>
+    <t>Reschedule appointment</t>
+  </si>
+  <si>
+    <t>{"newDate":"", "newTime":""}</t>
+  </si>
+  <si>
+    <t>/appointments/{appointmentId}/status</t>
+  </si>
+  <si>
+    <t>Update appointment status</t>
+  </si>
+  <si>
+    <t>{"status":"completed"}</t>
+  </si>
+  <si>
+    <t>/appointments/{appointmentId}</t>
+  </si>
+  <si>
+    <t>Get appointment details</t>
+  </si>
+  <si>
+    <t>Path Variable: appointmentId</t>
+  </si>
+  <si>
+    <t>/appointments/doctor/{doctorId}/calendar</t>
+  </si>
+  <si>
+    <t>Doctor calendar view</t>
+  </si>
+  <si>
+    <t>/appointments/patient/{patientId}/calendar</t>
+  </si>
+  <si>
+    <t>Patient calendar view</t>
+  </si>
+  <si>
+    <t>Update user profile</t>
+  </si>
+  <si>
+    <t>{"name":"", "phone":""}</t>
+  </si>
+  <si>
+    <t>Delete user</t>
+  </si>
+  <si>
+    <t>Path Variable: id</t>
+  </si>
+  <si>
+    <t>/user/{id}/role</t>
+  </si>
+  <si>
+    <t>Change role</t>
+  </si>
+  <si>
+    <t>{"role":"ADMIN"}</t>
+  </si>
+  <si>
+    <t>/admin/create-user</t>
+  </si>
+  <si>
+    <t>Create new system user</t>
+  </si>
+  <si>
+    <t>{"name":"", "email":"", "role":""}</t>
+  </si>
+  <si>
+    <t>Update admin</t>
+  </si>
+  <si>
+    <t>{"name":"", "email":""}</t>
+  </si>
+  <si>
+    <t>Delete admin</t>
+  </si>
+  <si>
+    <t>/admin/analytics/overview</t>
+  </si>
+  <si>
+    <t>System overview metrics</t>
+  </si>
+  <si>
+    <t>/admin/analytics/appointments</t>
+  </si>
+  <si>
+    <t>Appointment statistics</t>
+  </si>
+  <si>
+    <t>/admin/analytics/doctor-performance</t>
+  </si>
+  <si>
+    <t>Doctor performance metrics</t>
+  </si>
+  <si>
+    <t>/medical-records/{recordId}</t>
+  </si>
+  <si>
+    <t>Get medical record</t>
+  </si>
+  <si>
+    <t>Path Variable: recordId</t>
+  </si>
+  <si>
+    <t>Update medical record</t>
+  </si>
+  <si>
+    <t>{"notes":"", "type":""}</t>
+  </si>
+  <si>
+    <t>Delete medical record</t>
+  </si>
+  <si>
+    <t>/medical-records/{patientId}/prescriptions</t>
+  </si>
+  <si>
+    <t>Upload prescription</t>
+  </si>
+  <si>
+    <t>{"file":"base64"}</t>
+  </si>
+  <si>
+    <t>List prescriptions</t>
+  </si>
+  <si>
+    <t>/medical-records/{patientId}/lab-reports</t>
+  </si>
+  <si>
+    <t>Upload lab report</t>
+  </si>
+  <si>
+    <t>List lab reports</t>
+  </si>
+  <si>
+    <t>Notifications</t>
+  </si>
+  <si>
+    <t>/notifications/send</t>
+  </si>
+  <si>
+    <t>Send notification</t>
+  </si>
+  <si>
+    <t>{"userId":"", "message":""}</t>
+  </si>
+  <si>
+    <t>/notifications/user/{userId}</t>
+  </si>
+  <si>
+    <t>Get notifications</t>
+  </si>
+  <si>
+    <t>Path Variable: userId</t>
+  </si>
+  <si>
+    <t>/notifications/settings/{userId}</t>
+  </si>
+  <si>
+    <t>Update notification settings</t>
+  </si>
+  <si>
+    <t>{"email":true, "sms":false}</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>In-Work</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -65,8 +591,59 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="29">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Mongolian Baiti"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -223,13 +800,44 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14.05"/>
+      <color rgb="FF1F2937"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F46E5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -418,12 +1026,129 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="18">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFAAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFAAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -544,141 +1269,215 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -733,7 +1532,88 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="20">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <u val="none"/>
+        <color rgb="FF1D4ED8"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.6"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <i val="0"/>
+        <color rgb="FF065F46"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD1FAE5"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <i val="0"/>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -927,33 +1807,847 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="9"/>
+      <tableStyleElement type="headerRow" dxfId="8"/>
+      <tableStyleElement type="totalRow" dxfId="7"/>
+      <tableStyleElement type="firstColumn" dxfId="6"/>
+      <tableStyleElement type="lastColumn" dxfId="5"/>
+      <tableStyleElement type="firstRowStripe" dxfId="4"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="3"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="19"/>
+      <tableStyleElement type="totalRow" dxfId="18"/>
+      <tableStyleElement type="firstRowStripe" dxfId="17"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="16"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="15"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="14"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="13"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="12"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="11"/>
+      <tableStyleElement type="pageFieldValues" dxfId="10"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="00B2EC0A"/>
+      <color rgb="0093E312"/>
+      <color rgb="00D1FAE5"/>
+      <color rgb="00065F46"/>
+      <color rgb="001D4ED8"/>
+      <color rgb="00991B1B"/>
+      <color rgb="00FEE2E2"/>
+      <color rgb="004F46E5"/>
+      <color rgb="00FFFFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'API''s Pending'!$B$46</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Count</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr/>
+          <c:explosion val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'API''s Pending'!$A$47:$A$49</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Pending</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>In-Work</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Completed</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'API''s Pending'!$B$47:$B$49</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr lang="en-US"/>
+      </a:pPr>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="10082">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="bg1"/>
+        </a:solidFill>
+      </a:ln>
+      <a:effectLst/>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="90200"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="1" kern="1200" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1889125</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="6673850" y="9499600"/>
+        <a:ext cx="5445125" cy="2743200"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1218,6 +2912,7 @@
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="46.4285714285714" customWidth="1"/>
+    <col min="2" max="2" width="43.1428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1232,7 +2927,7 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="27" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1261,9 +2956,435 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
-  <sheetData/>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="24.4285714285714" customWidth="1"/>
+    <col min="2" max="2" width="38.4285714285714" style="10" customWidth="1"/>
+    <col min="3" max="3" width="14.7142857142857" style="11" customWidth="1"/>
+    <col min="4" max="4" width="140.857142857143" style="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="9" customFormat="1" ht="15.75" spans="1:5">
+      <c r="A1" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="15"/>
+    </row>
+    <row r="2" ht="31.5" spans="1:4">
+      <c r="A2" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" spans="1:4">
+      <c r="A3" s="16"/>
+      <c r="B3" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" spans="1:4">
+      <c r="A4" s="16"/>
+      <c r="B4" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" spans="1:4">
+      <c r="A5" s="16"/>
+      <c r="B5" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" spans="1:4">
+      <c r="A6" s="16"/>
+      <c r="B6" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" spans="1:4">
+      <c r="A7" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" spans="1:4">
+      <c r="A8" s="16"/>
+      <c r="B8" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75" spans="1:4">
+      <c r="A9" s="16"/>
+      <c r="B9" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75" spans="1:4">
+      <c r="A10" s="16"/>
+      <c r="B10" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" spans="1:4">
+      <c r="A11" s="16"/>
+      <c r="B11" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" spans="1:4">
+      <c r="A12" s="16"/>
+      <c r="B12" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" spans="1:4">
+      <c r="A13" s="16"/>
+      <c r="B13" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" spans="1:4">
+      <c r="A14" s="16"/>
+      <c r="B14" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" ht="15.75" spans="1:4">
+      <c r="A15" s="16"/>
+      <c r="B15" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" ht="31.5" spans="1:4">
+      <c r="A16" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" ht="15.75" spans="1:4">
+      <c r="A17" s="16"/>
+      <c r="B17" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" spans="1:4">
+      <c r="A18" s="16"/>
+      <c r="B18" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" ht="15.75" spans="1:4">
+      <c r="A19" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" spans="1:4">
+      <c r="A20" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" spans="1:4">
+      <c r="A21" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" spans="1:4">
+      <c r="A22" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" spans="1:4">
+      <c r="A23" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" spans="1:4">
+      <c r="A24" s="21"/>
+      <c r="B24" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" spans="1:4">
+      <c r="A25" s="22"/>
+      <c r="B25" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" spans="1:4">
+      <c r="A26" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" spans="1:4">
+      <c r="A27" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="34" ht="18" spans="1:2">
+      <c r="A34" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="23"/>
+    </row>
+    <row r="35" ht="18" spans="1:4">
+      <c r="A35" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="25">
+        <f>COUNTA(B2:B27)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="26"/>
+      <c r="D35"/>
+    </row>
+    <row r="36" ht="18" spans="1:4">
+      <c r="A36" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="25">
+        <f>COUNTIF(C2:C28,"POST")</f>
+        <v>12</v>
+      </c>
+      <c r="C36"/>
+      <c r="D36"/>
+    </row>
+    <row r="37" ht="18" spans="1:2">
+      <c r="A37" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="25">
+        <f>COUNTIF(C2:C27,"GET")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" ht="18" spans="1:2">
+      <c r="A38" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="B38" s="25">
+        <f>COUNTIF(C2:C28,"DELETE")</f>
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A7:A15"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="A26:A27"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C$1:C$1048576">
+    <cfRule type="cellIs" dxfId="0" priority="3" stopIfTrue="1" operator="equal">
+      <formula>"GET"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="equal">
+      <formula>"POST"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"DELETE"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C34 C37:C1048576">
+      <formula1>"GET,PUT,POST,DELETE,PATCH"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1272,10 +3393,972 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
-  <sheetData/>
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr defaultColWidth="42.4285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="15.1428571428571" style="1" customWidth="1"/>
+    <col min="2" max="2" width="40.2857142857143" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85714285714286" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42857142857143" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85714285714286" style="1" customWidth="1"/>
+    <col min="7" max="7" width="44.8571428571429" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="42.4285714285714" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="5"/>
+      <c r="B3" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="5"/>
+      <c r="B4" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="6"/>
+      <c r="B5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" ht="30" spans="1:7">
+      <c r="A6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="5"/>
+      <c r="B7" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="5"/>
+      <c r="B8" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="5"/>
+      <c r="B9" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="5"/>
+      <c r="B10" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="5"/>
+      <c r="B11" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="5"/>
+      <c r="B12" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="5"/>
+      <c r="B14" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="5"/>
+      <c r="B15" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="5"/>
+      <c r="B16" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="6"/>
+      <c r="B17" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" ht="30" spans="1:7">
+      <c r="A18" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="5"/>
+      <c r="B19" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="5"/>
+      <c r="B20" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="5"/>
+      <c r="B21" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="5"/>
+      <c r="B22" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="6"/>
+      <c r="B23" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="5"/>
+      <c r="B25" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="6"/>
+      <c r="B26" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="5"/>
+      <c r="B28" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="5"/>
+      <c r="B29" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="5"/>
+      <c r="B30" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="5"/>
+      <c r="B31" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="6"/>
+      <c r="B32" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="5"/>
+      <c r="B34" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="5"/>
+      <c r="B35" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="5"/>
+      <c r="B36" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="5"/>
+      <c r="B37" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="5"/>
+      <c r="B38" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="6"/>
+      <c r="B39" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="5"/>
+      <c r="B41" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="6"/>
+      <c r="B42" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B47" s="8">
+        <f>COUNTIF(D2:D42,"PENDING")</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B48" s="8">
+        <f>COUNTIF(D2:D42,"IN-WORK")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B49" s="8">
+        <f>COUNTIF(D2:D42,"COMPLETED")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="A13:A17"/>
+    <mergeCell ref="A18:A23"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="A33:A39"/>
+    <mergeCell ref="A40:A42"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 D2:D42 D43:D1048576">
+      <formula1>"PENDING,IN-Work,COMPLETED"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Bugs.xlsx and Helper.xlsx
</commit_message>
<xml_diff>
--- a/Helper.xlsx
+++ b/Helper.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" activeTab="2"/>
+    <workbookView windowWidth="23040" windowHeight="8280" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="180">
   <si>
     <t>Command to connect localhost to internet URL</t>
   </si>
@@ -260,6 +260,9 @@
     <t>Status</t>
   </si>
   <si>
+    <t>Method</t>
+  </si>
+  <si>
     <t>Start Date</t>
   </si>
   <si>
@@ -317,6 +320,9 @@
     <t>Update doctor profile</t>
   </si>
   <si>
+    <t>PUT</t>
+  </si>
+  <si>
     <t>{"name":"", "specialization":"", "experience":""}</t>
   </si>
   <si>
@@ -366,6 +372,9 @@
   </si>
   <si>
     <t>Update patient info</t>
+  </si>
+  <si>
+    <t>IN-Work</t>
   </si>
   <si>
     <t>{"name":"", "age":""}</t>
@@ -591,7 +600,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -603,13 +612,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1269,133 +1271,133 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1409,75 +1411,75 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1956,10 +1958,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>41</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2021,6 +2023,11 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext uri="{0b15fc19-7d7d-44ad-8c2d-2c3a37ce22c3}">
+        <chartProps xmlns="https://web.wps.cn/et/2018/main" chartId="{b567f7a2-c3b7-4457-8b0c-60487b402663}"/>
+      </c:ext>
+    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2619,13 +2626,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>25400</xdr:colOff>
       <xdr:row>47</xdr:row>
       <xdr:rowOff>165100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>1889125</xdr:colOff>
       <xdr:row>62</xdr:row>
       <xdr:rowOff>50800</xdr:rowOff>
@@ -2636,8 +2643,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6673850" y="9499600"/>
-        <a:ext cx="5445125" cy="2743200"/>
+        <a:off x="7647305" y="8760460"/>
+        <a:ext cx="5547995" cy="2628900"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2909,10 +2916,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="46.4285714285714" customWidth="1"/>
-    <col min="2" max="2" width="43.1428571428571" customWidth="1"/>
+    <col min="1" max="1" width="46.4259259259259" customWidth="1"/>
+    <col min="2" max="2" width="43.1388888888889" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2923,7 +2930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="18.75" spans="1:2">
+    <row r="2" ht="18" spans="1:2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2957,15 +2964,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E38"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="24.4285714285714" customWidth="1"/>
-    <col min="2" max="2" width="38.4285714285714" style="10" customWidth="1"/>
-    <col min="3" max="3" width="14.7142857142857" style="11" customWidth="1"/>
-    <col min="4" max="4" width="140.857142857143" style="12" customWidth="1"/>
+    <col min="1" max="1" width="24.4259259259259" customWidth="1"/>
+    <col min="2" max="2" width="38.4259259259259" style="11" customWidth="1"/>
+    <col min="3" max="3" width="14.712962962963" style="1" customWidth="1"/>
+    <col min="4" max="4" width="140.861111111111" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="9" customFormat="1" ht="15.75" spans="1:5">
+    <row r="1" s="10" customFormat="1" ht="15.6" spans="1:5">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -2980,7 +2987,7 @@
       </c>
       <c r="E1" s="15"/>
     </row>
-    <row r="2" ht="31.5" spans="1:4">
+    <row r="2" ht="31.2" spans="1:4">
       <c r="A2" s="16" t="s">
         <v>12</v>
       </c>
@@ -2994,7 +3001,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" ht="15.75" spans="1:4">
+    <row r="3" ht="15.6" spans="1:4">
       <c r="A3" s="16"/>
       <c r="B3" s="17" t="s">
         <v>16</v>
@@ -3006,7 +3013,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:4">
+    <row r="4" ht="15.6" spans="1:4">
       <c r="A4" s="16"/>
       <c r="B4" s="17" t="s">
         <v>18</v>
@@ -3018,7 +3025,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" ht="15.75" spans="1:4">
+    <row r="5" ht="15.6" spans="1:4">
       <c r="A5" s="16"/>
       <c r="B5" s="17" t="s">
         <v>20</v>
@@ -3030,7 +3037,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" ht="15.75" spans="1:4">
+    <row r="6" ht="15.6" spans="1:4">
       <c r="A6" s="16"/>
       <c r="B6" s="17" t="s">
         <v>22</v>
@@ -3042,7 +3049,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" ht="15.75" spans="1:4">
+    <row r="7" ht="15.6" spans="1:4">
       <c r="A7" s="16" t="s">
         <v>24</v>
       </c>
@@ -3056,7 +3063,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" ht="15.75" spans="1:4">
+    <row r="8" ht="15.6" spans="1:4">
       <c r="A8" s="16"/>
       <c r="B8" s="17" t="s">
         <v>27</v>
@@ -3068,7 +3075,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" ht="15.75" spans="1:4">
+    <row r="9" ht="15.6" spans="1:4">
       <c r="A9" s="16"/>
       <c r="B9" s="17" t="s">
         <v>27</v>
@@ -3080,7 +3087,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" ht="15.75" spans="1:4">
+    <row r="10" ht="15.6" spans="1:4">
       <c r="A10" s="16"/>
       <c r="B10" s="17" t="s">
         <v>30</v>
@@ -3092,7 +3099,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" ht="15.75" spans="1:4">
+    <row r="11" ht="15.6" spans="1:4">
       <c r="A11" s="16"/>
       <c r="B11" s="17" t="s">
         <v>32</v>
@@ -3104,7 +3111,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" ht="15.75" spans="1:4">
+    <row r="12" ht="15.6" spans="1:4">
       <c r="A12" s="16"/>
       <c r="B12" s="17" t="s">
         <v>34</v>
@@ -3116,7 +3123,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" ht="15.75" spans="1:4">
+    <row r="13" ht="15.6" spans="1:4">
       <c r="A13" s="16"/>
       <c r="B13" s="17" t="s">
         <v>36</v>
@@ -3128,7 +3135,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" ht="15.75" spans="1:4">
+    <row r="14" ht="15.6" spans="1:4">
       <c r="A14" s="16"/>
       <c r="B14" s="17" t="s">
         <v>38</v>
@@ -3140,7 +3147,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" ht="15.75" spans="1:4">
+    <row r="15" ht="15.6" spans="1:4">
       <c r="A15" s="16"/>
       <c r="B15" s="17" t="s">
         <v>40</v>
@@ -3152,7 +3159,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" ht="31.5" spans="1:4">
+    <row r="16" ht="31.2" spans="1:4">
       <c r="A16" s="16" t="s">
         <v>41</v>
       </c>
@@ -3166,7 +3173,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" ht="15.75" spans="1:4">
+    <row r="17" ht="15.6" spans="1:4">
       <c r="A17" s="16"/>
       <c r="B17" s="17" t="s">
         <v>44</v>
@@ -3178,7 +3185,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" ht="15.75" spans="1:4">
+    <row r="18" ht="15.6" spans="1:4">
       <c r="A18" s="16"/>
       <c r="B18" s="17" t="s">
         <v>46</v>
@@ -3190,7 +3197,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" ht="15.75" spans="1:4">
+    <row r="19" ht="15.6" spans="1:4">
       <c r="A19" s="16" t="s">
         <v>48</v>
       </c>
@@ -3204,7 +3211,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" ht="15.75" spans="1:4">
+    <row r="20" ht="15.6" spans="1:4">
       <c r="A20" s="16" t="s">
         <v>48</v>
       </c>
@@ -3218,7 +3225,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" ht="15.75" spans="1:4">
+    <row r="21" ht="15.6" spans="1:4">
       <c r="A21" s="16" t="s">
         <v>51</v>
       </c>
@@ -3232,7 +3239,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" ht="15.75" spans="1:4">
+    <row r="22" ht="15.6" spans="1:4">
       <c r="A22" s="16" t="s">
         <v>51</v>
       </c>
@@ -3246,7 +3253,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:4">
+    <row r="23" ht="15.6" spans="1:4">
       <c r="A23" s="20" t="s">
         <v>54</v>
       </c>
@@ -3260,7 +3267,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" ht="15.75" spans="1:4">
+    <row r="24" ht="15.6" spans="1:4">
       <c r="A24" s="21"/>
       <c r="B24" s="17" t="s">
         <v>56</v>
@@ -3272,7 +3279,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" ht="15.75" spans="1:4">
+    <row r="25" ht="15.6" spans="1:4">
       <c r="A25" s="22"/>
       <c r="B25" s="17" t="s">
         <v>56</v>
@@ -3284,7 +3291,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" ht="15.75" spans="1:4">
+    <row r="26" ht="15.6" spans="1:4">
       <c r="A26" s="16" t="s">
         <v>57</v>
       </c>
@@ -3298,7 +3305,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" ht="15.75" spans="1:4">
+    <row r="27" ht="15.6" spans="1:4">
       <c r="A27" s="16" t="s">
         <v>57</v>
       </c>
@@ -3312,13 +3319,13 @@
         <v>61</v>
       </c>
     </row>
-    <row r="34" ht="18" spans="1:2">
+    <row r="34" ht="17.4" spans="1:2">
       <c r="A34" s="23" t="s">
         <v>62</v>
       </c>
       <c r="B34" s="23"/>
     </row>
-    <row r="35" ht="18" spans="1:4">
+    <row r="35" ht="17.4" spans="1:4">
       <c r="A35" s="24" t="s">
         <v>63</v>
       </c>
@@ -3329,7 +3336,7 @@
       <c r="C35" s="26"/>
       <c r="D35"/>
     </row>
-    <row r="36" ht="18" spans="1:4">
+    <row r="36" ht="17.4" spans="1:4">
       <c r="A36" s="24" t="s">
         <v>64</v>
       </c>
@@ -3340,7 +3347,7 @@
       <c r="C36"/>
       <c r="D36"/>
     </row>
-    <row r="37" ht="18" spans="1:2">
+    <row r="37" ht="17.4" spans="1:2">
       <c r="A37" s="24" t="s">
         <v>65</v>
       </c>
@@ -3349,7 +3356,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" ht="18" spans="1:2">
+    <row r="38" ht="17.4" spans="1:2">
       <c r="A38" s="24" t="s">
         <v>66</v>
       </c>
@@ -3393,20 +3400,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G49"/>
-  <sheetFormatPr defaultColWidth="42.4285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <dimension ref="A1:H49"/>
+  <sheetFormatPr defaultColWidth="42.4259259259259" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="15.1428571428571" style="1" customWidth="1"/>
-    <col min="2" max="2" width="40.2857142857143" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1388888888889" style="1" customWidth="1"/>
+    <col min="2" max="2" width="40.287037037037" style="1" customWidth="1"/>
     <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85714285714286" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42857142857143" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85714285714286" style="1" customWidth="1"/>
-    <col min="7" max="7" width="44.8571428571429" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="42.4285714285714" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.4259259259259" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.86111111111111" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42592592592593" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.86111111111111" style="1" customWidth="1"/>
+    <col min="8" max="8" width="44.8611111111111" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="42.4259259259259" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -3428,478 +3436,547 @@
       <c r="G1" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E2" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E2" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="F2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="6"/>
+      <c r="B3" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="5"/>
-      <c r="B3" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="6"/>
+      <c r="B4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="E4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="7"/>
+      <c r="B5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="5"/>
-      <c r="B4" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="6"/>
-      <c r="B5" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>76</v>
+      <c r="E5" s="5" t="s">
+        <v>14</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" ht="30" spans="1:7">
+        <v>77</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E6" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="F6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="6"/>
+      <c r="B7" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="5"/>
-      <c r="B7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="6"/>
+      <c r="B8" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="E8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="6"/>
+      <c r="B9" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="5"/>
-      <c r="B8" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="E9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="6"/>
+      <c r="B10" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="E10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="6"/>
+      <c r="B11" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G8" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="5"/>
-      <c r="B9" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" s="4" t="s">
+      <c r="E11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="6"/>
+      <c r="B12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="5"/>
-      <c r="B10" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="E12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="5"/>
-      <c r="B11" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="5"/>
-      <c r="B12" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E13" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="6"/>
+      <c r="B14" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="E14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="6"/>
+      <c r="B15" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G13" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="5"/>
-      <c r="B14" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="E15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="6"/>
+      <c r="B16" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="E16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="7"/>
+      <c r="B17" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="5"/>
-      <c r="B15" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="5"/>
-      <c r="B16" s="4" t="s">
+      <c r="E17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="6"/>
-      <c r="B17" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="18" ht="30" spans="1:7">
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E18" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E18" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="F18" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="6"/>
+      <c r="B19" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="5"/>
-      <c r="B19" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="6"/>
+      <c r="B20" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="E20" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="6"/>
+      <c r="B21" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="5"/>
-      <c r="B20" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E20" s="4" t="s">
+      <c r="E21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="6"/>
+      <c r="B22" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="E22" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="7"/>
+      <c r="B23" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G20" s="4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="5"/>
-      <c r="B21" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="5"/>
-      <c r="B22" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="6"/>
-      <c r="B23" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>76</v>
+      <c r="E23" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+        <v>77</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="3" t="s">
         <v>51</v>
       </c>
@@ -3907,436 +3984,493 @@
         <v>53</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E24" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="F24" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="5"/>
+        <v>77</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="6"/>
       <c r="B25" s="4" t="s">
         <v>53</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E25" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E25" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="F25" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="7"/>
+      <c r="B26" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G25" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="6"/>
-      <c r="B26" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>76</v>
+      <c r="E26" s="5" t="s">
+        <v>90</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
+        <v>77</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E27" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E27" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="F27" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" s="5"/>
+        <v>77</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" s="6"/>
       <c r="B28" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E28" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E28" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="F28" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="5"/>
+        <v>77</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="6"/>
       <c r="B29" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E29" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E29" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="F29" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="6"/>
+      <c r="B30" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G29" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="5"/>
-      <c r="B30" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="6"/>
+      <c r="B31" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="E31" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="7"/>
+      <c r="B32" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D32" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G30" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" s="5"/>
-      <c r="B31" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="6"/>
-      <c r="B32" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>76</v>
+      <c r="E32" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+        <v>77</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E33" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="E33" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="F33" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="6"/>
+      <c r="B34" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G33" s="4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" s="5"/>
-      <c r="B34" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C34" s="4" t="s">
+      <c r="E34" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="6"/>
+      <c r="B35" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="D34" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E34" s="4" t="s">
+      <c r="C35" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="E35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="6"/>
+      <c r="B36" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D36" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G34" s="4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35" s="5"/>
-      <c r="B35" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E35" s="4" t="s">
+      <c r="E36" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="6"/>
+      <c r="B37" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="E37" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="6"/>
+      <c r="B38" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D38" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G35" s="4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
-      <c r="A36" s="5"/>
-      <c r="B36" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E36" s="4" t="s">
+      <c r="E38" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="7"/>
+      <c r="B39" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D39" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="E39" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D40" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G36" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37" s="5"/>
-      <c r="B37" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E37" s="4" t="s">
+      <c r="E40" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="6"/>
+      <c r="B41" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D41" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="E41" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="7"/>
+      <c r="B42" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D42" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G37" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="5"/>
-      <c r="B38" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" s="6"/>
-      <c r="B39" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F40" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41" s="5"/>
-      <c r="B41" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
-      <c r="A42" s="6"/>
-      <c r="B42" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>76</v>
+      <c r="E42" s="5" t="s">
+        <v>90</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>172</v>
+        <v>77</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="7" t="s">
+      <c r="A46" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B46" s="7" t="s">
-        <v>173</v>
+      <c r="B46" s="8" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="B47" s="8">
+      <c r="A47" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B47" s="9">
         <f>COUNTIF(D2:D42,"PENDING")</f>
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="B48" s="8">
+      <c r="A48" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="B48" s="9">
         <f>COUNTIF(D2:D42,"IN-WORK")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B49" s="8">
+      <c r="A49" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B49" s="9">
         <f>COUNTIF(D2:D42,"COMPLETED")</f>
         <v>0</v>
       </c>
@@ -4352,9 +4486,12 @@
     <mergeCell ref="A33:A39"/>
     <mergeCell ref="A40:A42"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 D2:D42 D43:D1048576">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D$1:D$1048576">
       <formula1>"PENDING,IN-Work,COMPLETED"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E$1:E$1048576">
+      <formula1>"GET,PUT,POST,PATCH,DELETE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>